<commit_message>
Add Galaxy Z foldables and iPad (A16); remove Galaxy S26+; order /devices by line
- New device pages: Galaxy Z Fold8 Ultra, Z Fold7, Z Flip7, Z Fold6, Z Fold3
  and iPad (11th gen, A16), with specs (GSMArena / Apple) and credited
  Wikimedia Commons photos. The iPad page sells the store's own Shopify listing.
- Galaxy S26+ removed (not carried)
- /devices: sections by company and line (iPhone, Galaxy S & Note, Galaxy Z,
  Galaxy A, iPad), families newest first, models in the makers' order, with
  jump links; filters match the sections
- docs/shopify/new-products-2026-10-27.csv: the foldables ready to sell at the
  owner's prices, iPad mini 5 as a draft; price update adds iPad (A16) prices;
  master import file updated
- Device lists for search, AI answers and Tidio regenerated (58 devices)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/shopify/price-update-2026-10-27.xlsx
+++ b/docs/shopify/price-update-2026-10-27.xlsx
@@ -88,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -106,6 +106,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -471,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1729,6 +1732,161 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>Apple iPad 11th Generation WiFi 128GB</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="n">
+        <v>549</v>
+      </c>
+      <c r="D41" s="12" t="n">
+        <v>599</v>
+      </c>
+      <c r="E41" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>In stock</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>Owner: iPad 11th Gen Wi-Fi → $599</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>Apple iPad 11th Generation WiFi 128GB</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="n">
+        <v>549</v>
+      </c>
+      <c r="D42" s="12" t="n">
+        <v>599</v>
+      </c>
+      <c r="E42" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="F42" s="11" t="inlineStr">
+        <is>
+          <t>In stock</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr">
+        <is>
+          <t>Owner: iPad 11th Gen Wi-Fi → $599</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>Apple iPad 11th Generation WiFi 128GB</t>
+        </is>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="n">
+        <v>549</v>
+      </c>
+      <c r="D43" s="12" t="n">
+        <v>599</v>
+      </c>
+      <c r="E43" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>In stock</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>Owner: iPad 11th Gen Wi-Fi → $599</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>Apple iPad 11th Generation WiFi 128GB</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>Pink</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="n">
+        <v>549</v>
+      </c>
+      <c r="D44" s="12" t="n">
+        <v>599</v>
+      </c>
+      <c r="E44" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="F44" s="11" t="inlineStr">
+        <is>
+          <t>In stock</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>Owner: iPad 11th Gen Wi-Fi → $599</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>Apple iPad 11th Generation WiFi + Cellular 128GB</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>599</v>
+      </c>
+      <c r="D45" s="12" t="n">
+        <v>750</v>
+      </c>
+      <c r="E45" s="12" t="n">
+        <v>151</v>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>In stock</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>Owner: iPad 11th Gen Wi-Fi + Cellular → $750</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1741,7 +1899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1921,6 +2079,31 @@
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>In stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Apple iPad 11th Generation WiFi + Cellular 256GB</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="n">
+        <v>550</v>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Costs less than the 128GB Wi-Fi + Cellular ($750 after this update). Not on your note, so not changed — set its price in Shopify.</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>In stock</t>
         </is>
@@ -1938,7 +2121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4150,6 +4333,121 @@
         <v>1599</v>
       </c>
       <c r="E109" s="6" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Apple iPad 11th Generation WiFi 128GB</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>549</v>
+      </c>
+      <c r="D110" t="n">
+        <v>599</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Apple iPad 11th Generation WiFi 128GB</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>549</v>
+      </c>
+      <c r="D111" t="n">
+        <v>599</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Apple iPad 11th Generation WiFi 128GB</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>549</v>
+      </c>
+      <c r="D112" t="n">
+        <v>599</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Apple iPad 11th Generation WiFi 128GB</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Pink</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>549</v>
+      </c>
+      <c r="D113" t="n">
+        <v>599</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Apple iPad 11th Generation WiFi + Cellular 128GB</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>599</v>
+      </c>
+      <c r="D114" t="n">
+        <v>750</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E109"/>
@@ -4211,9 +4509,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>

</xml_diff>